<commit_message>
feat:added defined cost field in pricing page
</commit_message>
<xml_diff>
--- a/Tools_Data.xlsx
+++ b/Tools_Data.xlsx
@@ -16031,7 +16031,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J802"/>
+  <dimension ref="A1:J803"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="27.83203125" customWidth="1"/>
@@ -41709,9 +41709,41 @@
         <v>10</v>
       </c>
     </row>
+    <row r="803">
+      <c r="A803" t="str">
+        <v>1</v>
+      </c>
+      <c r="B803" t="str">
+        <v>Base Unit</v>
+      </c>
+      <c r="C803" t="str">
+        <v>1</v>
+      </c>
+      <c r="D803" t="str">
+        <v>Pullout Cabinet</v>
+      </c>
+      <c r="E803" t="str">
+        <v>1</v>
+      </c>
+      <c r="F803" t="str">
+        <v>B15</v>
+      </c>
+      <c r="G803" t="str">
+        <v>802</v>
+      </c>
+      <c r="H803" t="str">
+        <v>Test</v>
+      </c>
+      <c r="I803" t="str">
+        <v>0</v>
+      </c>
+      <c r="J803" t="str">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J802"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J803"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>